<commit_message>
Added merged + updated datasets
Updated temperature with NOAA data
Added back NAICS 311230
Added merged datasets
</commit_message>
<xml_diff>
--- a/final_data_pipeline/output/311221_elec_options.xlsx
+++ b/final_data_pipeline/output/311221_elec_options.xlsx
@@ -1116,7 +1116,7 @@
         <v>179</v>
       </c>
       <c r="AD2">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE2">
         <v>8000</v>
@@ -1211,7 +1211,7 @@
         <v>179</v>
       </c>
       <c r="AD3">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE3">
         <v>8000</v>
@@ -1309,7 +1309,7 @@
         <v>179</v>
       </c>
       <c r="AD4">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE4">
         <v>8000</v>
@@ -1407,7 +1407,7 @@
         <v>179</v>
       </c>
       <c r="AD5">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE5">
         <v>8000</v>
@@ -1505,7 +1505,7 @@
         <v>179</v>
       </c>
       <c r="AD6">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE6">
         <v>8000</v>
@@ -1603,7 +1603,7 @@
         <v>179</v>
       </c>
       <c r="AD7">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE7">
         <v>8000</v>
@@ -1701,7 +1701,7 @@
         <v>179</v>
       </c>
       <c r="AD8">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE8">
         <v>8000</v>
@@ -1799,7 +1799,7 @@
         <v>179</v>
       </c>
       <c r="AD9">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE9">
         <v>8000</v>
@@ -1897,7 +1897,7 @@
         <v>179</v>
       </c>
       <c r="AD10">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE10">
         <v>8000</v>
@@ -1992,7 +1992,7 @@
         <v>179</v>
       </c>
       <c r="AD11">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE11">
         <v>8000</v>
@@ -2090,7 +2090,7 @@
         <v>179</v>
       </c>
       <c r="AD12">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE12">
         <v>8000</v>
@@ -2188,7 +2188,7 @@
         <v>179</v>
       </c>
       <c r="AD13">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE13">
         <v>8000</v>
@@ -2283,7 +2283,7 @@
         <v>179</v>
       </c>
       <c r="AD14">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE14">
         <v>8000</v>
@@ -2378,7 +2378,7 @@
         <v>179</v>
       </c>
       <c r="AD15">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE15">
         <v>8000</v>
@@ -2473,7 +2473,7 @@
         <v>179</v>
       </c>
       <c r="AD16">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE16">
         <v>8000</v>
@@ -2568,7 +2568,7 @@
         <v>179</v>
       </c>
       <c r="AD17">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE17">
         <v>8000</v>
@@ -2663,7 +2663,7 @@
         <v>179</v>
       </c>
       <c r="AD18">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE18">
         <v>8000</v>
@@ -2761,7 +2761,7 @@
         <v>179</v>
       </c>
       <c r="AD19">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE19">
         <v>8000</v>
@@ -2859,7 +2859,7 @@
         <v>179</v>
       </c>
       <c r="AD20">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE20">
         <v>8000</v>
@@ -2957,7 +2957,7 @@
         <v>179</v>
       </c>
       <c r="AD21">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE21">
         <v>8000</v>
@@ -3055,7 +3055,7 @@
         <v>179</v>
       </c>
       <c r="AD22">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE22">
         <v>8000</v>
@@ -3150,7 +3150,7 @@
         <v>179</v>
       </c>
       <c r="AD23">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE23">
         <v>8000</v>
@@ -3248,7 +3248,7 @@
         <v>179</v>
       </c>
       <c r="AD24">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE24">
         <v>8000</v>
@@ -3346,7 +3346,7 @@
         <v>179</v>
       </c>
       <c r="AD25">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE25">
         <v>8000</v>
@@ -3441,7 +3441,7 @@
         <v>179</v>
       </c>
       <c r="AD26">
-        <v>10</v>
+        <v>1.791666666666668</v>
       </c>
       <c r="AE26">
         <v>8000</v>
@@ -4504,7 +4504,7 @@
         <v>179</v>
       </c>
       <c r="AD37">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE37">
         <v>8000</v>
@@ -4599,7 +4599,7 @@
         <v>179</v>
       </c>
       <c r="AD38">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE38">
         <v>8000</v>
@@ -4694,7 +4694,7 @@
         <v>179</v>
       </c>
       <c r="AD39">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE39">
         <v>8000</v>
@@ -4792,7 +4792,7 @@
         <v>179</v>
       </c>
       <c r="AD40">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE40">
         <v>8000</v>
@@ -4890,7 +4890,7 @@
         <v>179</v>
       </c>
       <c r="AD41">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE41">
         <v>8000</v>
@@ -4988,7 +4988,7 @@
         <v>179</v>
       </c>
       <c r="AD42">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE42">
         <v>8000</v>
@@ -5086,7 +5086,7 @@
         <v>179</v>
       </c>
       <c r="AD43">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE43">
         <v>8000</v>
@@ -5184,7 +5184,7 @@
         <v>179</v>
       </c>
       <c r="AD44">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE44">
         <v>8000</v>
@@ -5282,7 +5282,7 @@
         <v>179</v>
       </c>
       <c r="AD45">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE45">
         <v>8000</v>
@@ -5380,7 +5380,7 @@
         <v>179</v>
       </c>
       <c r="AD46">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE46">
         <v>8000</v>
@@ -5478,7 +5478,7 @@
         <v>179</v>
       </c>
       <c r="AD47">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE47">
         <v>8000</v>
@@ -5573,7 +5573,7 @@
         <v>179</v>
       </c>
       <c r="AD48">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE48">
         <v>8000</v>
@@ -5668,7 +5668,7 @@
         <v>179</v>
       </c>
       <c r="AD49">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE49">
         <v>8000</v>
@@ -5763,7 +5763,7 @@
         <v>179</v>
       </c>
       <c r="AD50">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE50">
         <v>8000</v>
@@ -5858,7 +5858,7 @@
         <v>179</v>
       </c>
       <c r="AD51">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE51">
         <v>8000</v>
@@ -5953,7 +5953,7 @@
         <v>179</v>
       </c>
       <c r="AD52">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE52">
         <v>8000</v>
@@ -6048,7 +6048,7 @@
         <v>179</v>
       </c>
       <c r="AD53">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE53">
         <v>8000</v>
@@ -6146,7 +6146,7 @@
         <v>179</v>
       </c>
       <c r="AD54">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE54">
         <v>8000</v>
@@ -6244,7 +6244,7 @@
         <v>179</v>
       </c>
       <c r="AD55">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE55">
         <v>8000</v>
@@ -6342,7 +6342,7 @@
         <v>179</v>
       </c>
       <c r="AD56">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE56">
         <v>8000</v>
@@ -6440,7 +6440,7 @@
         <v>179</v>
       </c>
       <c r="AD57">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE57">
         <v>8000</v>
@@ -6538,7 +6538,7 @@
         <v>179</v>
       </c>
       <c r="AD58">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE58">
         <v>8000</v>
@@ -6633,7 +6633,7 @@
         <v>179</v>
       </c>
       <c r="AD59">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE59">
         <v>8000</v>
@@ -6731,7 +6731,7 @@
         <v>179</v>
       </c>
       <c r="AD60">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE60">
         <v>8000</v>
@@ -6829,7 +6829,7 @@
         <v>179</v>
       </c>
       <c r="AD61">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE61">
         <v>8000</v>
@@ -6924,7 +6924,7 @@
         <v>179</v>
       </c>
       <c r="AD62">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE62">
         <v>8000</v>
@@ -7022,7 +7022,7 @@
         <v>179</v>
       </c>
       <c r="AD63">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE63">
         <v>8000</v>
@@ -7120,7 +7120,7 @@
         <v>179</v>
       </c>
       <c r="AD64">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE64">
         <v>8000</v>
@@ -7215,7 +7215,7 @@
         <v>179</v>
       </c>
       <c r="AD65">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE65">
         <v>8000</v>
@@ -7310,7 +7310,7 @@
         <v>179</v>
       </c>
       <c r="AD66">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE66">
         <v>8000</v>
@@ -7405,7 +7405,7 @@
         <v>179</v>
       </c>
       <c r="AD67">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE67">
         <v>8000</v>
@@ -7500,7 +7500,7 @@
         <v>179</v>
       </c>
       <c r="AD68">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE68">
         <v>8000</v>
@@ -7598,7 +7598,7 @@
         <v>179</v>
       </c>
       <c r="AD69">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE69">
         <v>8000</v>
@@ -7696,7 +7696,7 @@
         <v>179</v>
       </c>
       <c r="AD70">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE70">
         <v>8000</v>
@@ -7794,7 +7794,7 @@
         <v>179</v>
       </c>
       <c r="AD71">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE71">
         <v>8000</v>
@@ -7889,7 +7889,7 @@
         <v>179</v>
       </c>
       <c r="AD72">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE72">
         <v>8000</v>
@@ -7987,7 +7987,7 @@
         <v>179</v>
       </c>
       <c r="AD73">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE73">
         <v>8000</v>
@@ -8085,7 +8085,7 @@
         <v>179</v>
       </c>
       <c r="AD74">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE74">
         <v>8000</v>
@@ -8183,7 +8183,7 @@
         <v>179</v>
       </c>
       <c r="AD75">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE75">
         <v>8000</v>
@@ -8281,7 +8281,7 @@
         <v>179</v>
       </c>
       <c r="AD76">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE76">
         <v>8000</v>
@@ -8379,7 +8379,7 @@
         <v>179</v>
       </c>
       <c r="AD77">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE77">
         <v>8000</v>
@@ -8477,7 +8477,7 @@
         <v>179</v>
       </c>
       <c r="AD78">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE78">
         <v>8000</v>
@@ -8575,7 +8575,7 @@
         <v>179</v>
       </c>
       <c r="AD79">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE79">
         <v>8000</v>
@@ -8670,7 +8670,7 @@
         <v>179</v>
       </c>
       <c r="AD80">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE80">
         <v>8000</v>
@@ -8765,7 +8765,7 @@
         <v>179</v>
       </c>
       <c r="AD81">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE81">
         <v>8000</v>
@@ -8863,7 +8863,7 @@
         <v>179</v>
       </c>
       <c r="AD82">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE82">
         <v>8000</v>
@@ -8961,7 +8961,7 @@
         <v>179</v>
       </c>
       <c r="AD83">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE83">
         <v>8000</v>
@@ -9059,7 +9059,7 @@
         <v>179</v>
       </c>
       <c r="AD84">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE84">
         <v>8000</v>
@@ -9157,7 +9157,7 @@
         <v>179</v>
       </c>
       <c r="AD85">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE85">
         <v>8000</v>
@@ -9255,7 +9255,7 @@
         <v>179</v>
       </c>
       <c r="AD86">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE86">
         <v>8000</v>
@@ -9353,7 +9353,7 @@
         <v>179</v>
       </c>
       <c r="AD87">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE87">
         <v>8000</v>
@@ -9448,7 +9448,7 @@
         <v>179</v>
       </c>
       <c r="AD88">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE88">
         <v>8000</v>
@@ -9543,7 +9543,7 @@
         <v>179</v>
       </c>
       <c r="AD89">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE89">
         <v>8000</v>
@@ -9638,7 +9638,7 @@
         <v>179</v>
       </c>
       <c r="AD90">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE90">
         <v>8000</v>
@@ -9733,7 +9733,7 @@
         <v>179</v>
       </c>
       <c r="AD91">
-        <v>10</v>
+        <v>19.79629629629628</v>
       </c>
       <c r="AE91">
         <v>8000</v>
@@ -9831,7 +9831,7 @@
         <v>179</v>
       </c>
       <c r="AD92">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE92">
         <v>8000</v>
@@ -9929,7 +9929,7 @@
         <v>179</v>
       </c>
       <c r="AD93">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE93">
         <v>8000</v>
@@ -10027,7 +10027,7 @@
         <v>179</v>
       </c>
       <c r="AD94">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE94">
         <v>8000</v>
@@ -10125,7 +10125,7 @@
         <v>179</v>
       </c>
       <c r="AD95">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE95">
         <v>8000</v>
@@ -10223,7 +10223,7 @@
         <v>179</v>
       </c>
       <c r="AD96">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE96">
         <v>8000</v>
@@ -10321,7 +10321,7 @@
         <v>179</v>
       </c>
       <c r="AD97">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE97">
         <v>8000</v>
@@ -10419,7 +10419,7 @@
         <v>179</v>
       </c>
       <c r="AD98">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE98">
         <v>8000</v>
@@ -10517,7 +10517,7 @@
         <v>179</v>
       </c>
       <c r="AD99">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE99">
         <v>8000</v>
@@ -10615,7 +10615,7 @@
         <v>179</v>
       </c>
       <c r="AD100">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE100">
         <v>8000</v>
@@ -10713,7 +10713,7 @@
         <v>179</v>
       </c>
       <c r="AD101">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE101">
         <v>8000</v>
@@ -10808,7 +10808,7 @@
         <v>179</v>
       </c>
       <c r="AD102">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE102">
         <v>8000</v>
@@ -10906,7 +10906,7 @@
         <v>179</v>
       </c>
       <c r="AD103">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE103">
         <v>8000</v>
@@ -11001,7 +11001,7 @@
         <v>179</v>
       </c>
       <c r="AD104">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE104">
         <v>8000</v>
@@ -11096,7 +11096,7 @@
         <v>179</v>
       </c>
       <c r="AD105">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE105">
         <v>8000</v>
@@ -11191,7 +11191,7 @@
         <v>179</v>
       </c>
       <c r="AD106">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE106">
         <v>8000</v>
@@ -11289,7 +11289,7 @@
         <v>179</v>
       </c>
       <c r="AD107">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE107">
         <v>8000</v>
@@ -11384,7 +11384,7 @@
         <v>179</v>
       </c>
       <c r="AD108">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE108">
         <v>8000</v>
@@ -11479,7 +11479,7 @@
         <v>179</v>
       </c>
       <c r="AD109">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE109">
         <v>8000</v>
@@ -11577,7 +11577,7 @@
         <v>179</v>
       </c>
       <c r="AD110">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE110">
         <v>8000</v>
@@ -11672,7 +11672,7 @@
         <v>179</v>
       </c>
       <c r="AD111">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE111">
         <v>8000</v>
@@ -11770,7 +11770,7 @@
         <v>179</v>
       </c>
       <c r="AD112">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE112">
         <v>8000</v>
@@ -11865,7 +11865,7 @@
         <v>179</v>
       </c>
       <c r="AD113">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE113">
         <v>8000</v>
@@ -11960,7 +11960,7 @@
         <v>179</v>
       </c>
       <c r="AD114">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE114">
         <v>8000</v>
@@ -12055,7 +12055,7 @@
         <v>179</v>
       </c>
       <c r="AD115">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE115">
         <v>8000</v>
@@ -12150,7 +12150,7 @@
         <v>179</v>
       </c>
       <c r="AD116">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE116">
         <v>8000</v>
@@ -12245,7 +12245,7 @@
         <v>179</v>
       </c>
       <c r="AD117">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE117">
         <v>8000</v>
@@ -12340,7 +12340,7 @@
         <v>179</v>
       </c>
       <c r="AD118">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE118">
         <v>8000</v>
@@ -12435,7 +12435,7 @@
         <v>179</v>
       </c>
       <c r="AD119">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE119">
         <v>8000</v>
@@ -12533,7 +12533,7 @@
         <v>179</v>
       </c>
       <c r="AD120">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE120">
         <v>8000</v>
@@ -12631,7 +12631,7 @@
         <v>179</v>
       </c>
       <c r="AD121">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE121">
         <v>8000</v>
@@ -12729,7 +12729,7 @@
         <v>179</v>
       </c>
       <c r="AD122">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE122">
         <v>8000</v>
@@ -12827,7 +12827,7 @@
         <v>179</v>
       </c>
       <c r="AD123">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE123">
         <v>8000</v>
@@ -12925,7 +12925,7 @@
         <v>179</v>
       </c>
       <c r="AD124">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE124">
         <v>8000</v>
@@ -13023,7 +13023,7 @@
         <v>179</v>
       </c>
       <c r="AD125">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE125">
         <v>8000</v>
@@ -13124,7 +13124,7 @@
         <v>179</v>
       </c>
       <c r="AD126">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE126">
         <v>8000</v>
@@ -13225,7 +13225,7 @@
         <v>179</v>
       </c>
       <c r="AD127">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE127">
         <v>8000</v>
@@ -13326,7 +13326,7 @@
         <v>179</v>
       </c>
       <c r="AD128">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE128">
         <v>8000</v>
@@ -13427,7 +13427,7 @@
         <v>179</v>
       </c>
       <c r="AD129">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE129">
         <v>8000</v>
@@ -13525,7 +13525,7 @@
         <v>179</v>
       </c>
       <c r="AD130">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE130">
         <v>8000</v>
@@ -14104,7 +14104,7 @@
         <v>179</v>
       </c>
       <c r="AD136">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE136">
         <v>8000</v>
@@ -14202,7 +14202,7 @@
         <v>179</v>
       </c>
       <c r="AD137">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE137">
         <v>8000</v>
@@ -14300,7 +14300,7 @@
         <v>179</v>
       </c>
       <c r="AD138">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE138">
         <v>8000</v>
@@ -14398,7 +14398,7 @@
         <v>179</v>
       </c>
       <c r="AD139">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE139">
         <v>8000</v>
@@ -14496,7 +14496,7 @@
         <v>179</v>
       </c>
       <c r="AD140">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE140">
         <v>8000</v>
@@ -14594,7 +14594,7 @@
         <v>179</v>
       </c>
       <c r="AD141">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE141">
         <v>8000</v>
@@ -14692,7 +14692,7 @@
         <v>179</v>
       </c>
       <c r="AD142">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE142">
         <v>8000</v>
@@ -14790,7 +14790,7 @@
         <v>179</v>
       </c>
       <c r="AD143">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE143">
         <v>8000</v>
@@ -14888,7 +14888,7 @@
         <v>179</v>
       </c>
       <c r="AD144">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE144">
         <v>8000</v>
@@ -14986,7 +14986,7 @@
         <v>179</v>
       </c>
       <c r="AD145">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE145">
         <v>8000</v>
@@ -15084,7 +15084,7 @@
         <v>179</v>
       </c>
       <c r="AD146">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE146">
         <v>8000</v>
@@ -15182,7 +15182,7 @@
         <v>179</v>
       </c>
       <c r="AD147">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE147">
         <v>8000</v>
@@ -15280,7 +15280,7 @@
         <v>179</v>
       </c>
       <c r="AD148">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE148">
         <v>8000</v>
@@ -15378,7 +15378,7 @@
         <v>179</v>
       </c>
       <c r="AD149">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE149">
         <v>8000</v>
@@ -15476,7 +15476,7 @@
         <v>179</v>
       </c>
       <c r="AD150">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE150">
         <v>8000</v>
@@ -15574,7 +15574,7 @@
         <v>179</v>
       </c>
       <c r="AD151">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE151">
         <v>8000</v>
@@ -15672,7 +15672,7 @@
         <v>179</v>
       </c>
       <c r="AD152">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE152">
         <v>8000</v>
@@ -15767,7 +15767,7 @@
         <v>179</v>
       </c>
       <c r="AD153">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE153">
         <v>8000</v>
@@ -15865,7 +15865,7 @@
         <v>179</v>
       </c>
       <c r="AD154">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE154">
         <v>8000</v>
@@ -15960,7 +15960,7 @@
         <v>179</v>
       </c>
       <c r="AD155">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE155">
         <v>8000</v>
@@ -16055,7 +16055,7 @@
         <v>179</v>
       </c>
       <c r="AD156">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE156">
         <v>8000</v>
@@ -16153,7 +16153,7 @@
         <v>179</v>
       </c>
       <c r="AD157">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE157">
         <v>8000</v>
@@ -16251,7 +16251,7 @@
         <v>179</v>
       </c>
       <c r="AD158">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE158">
         <v>8000</v>
@@ -16349,7 +16349,7 @@
         <v>179</v>
       </c>
       <c r="AD159">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE159">
         <v>8000</v>
@@ -16447,7 +16447,7 @@
         <v>179</v>
       </c>
       <c r="AD160">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE160">
         <v>8000</v>
@@ -16542,7 +16542,7 @@
         <v>179</v>
       </c>
       <c r="AD161">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE161">
         <v>8000</v>
@@ -16637,7 +16637,7 @@
         <v>179</v>
       </c>
       <c r="AD162">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE162">
         <v>8000</v>
@@ -16732,7 +16732,7 @@
         <v>179</v>
       </c>
       <c r="AD163">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE163">
         <v>8000</v>
@@ -16827,7 +16827,7 @@
         <v>179</v>
       </c>
       <c r="AD164">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE164">
         <v>8000</v>
@@ -16922,7 +16922,7 @@
         <v>179</v>
       </c>
       <c r="AD165">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE165">
         <v>8000</v>
@@ -17017,7 +17017,7 @@
         <v>179</v>
       </c>
       <c r="AD166">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE166">
         <v>8000</v>
@@ -17112,7 +17112,7 @@
         <v>179</v>
       </c>
       <c r="AD167">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE167">
         <v>8000</v>
@@ -17207,7 +17207,7 @@
         <v>179</v>
       </c>
       <c r="AD168">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE168">
         <v>8000</v>
@@ -17302,7 +17302,7 @@
         <v>179</v>
       </c>
       <c r="AD169">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE169">
         <v>8000</v>
@@ -17397,7 +17397,7 @@
         <v>179</v>
       </c>
       <c r="AD170">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE170">
         <v>8000</v>
@@ -17492,7 +17492,7 @@
         <v>179</v>
       </c>
       <c r="AD171">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE171">
         <v>8000</v>
@@ -17587,7 +17587,7 @@
         <v>179</v>
       </c>
       <c r="AD172">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE172">
         <v>8000</v>
@@ -17685,7 +17685,7 @@
         <v>179</v>
       </c>
       <c r="AD173">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE173">
         <v>8000</v>
@@ -17783,7 +17783,7 @@
         <v>179</v>
       </c>
       <c r="AD174">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE174">
         <v>8000</v>
@@ -17881,7 +17881,7 @@
         <v>179</v>
       </c>
       <c r="AD175">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE175">
         <v>8000</v>
@@ -17979,7 +17979,7 @@
         <v>179</v>
       </c>
       <c r="AD176">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE176">
         <v>8000</v>
@@ -18077,7 +18077,7 @@
         <v>179</v>
       </c>
       <c r="AD177">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE177">
         <v>8000</v>
@@ -18172,7 +18172,7 @@
         <v>179</v>
       </c>
       <c r="AD178">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE178">
         <v>8000</v>
@@ -18267,7 +18267,7 @@
         <v>179</v>
       </c>
       <c r="AD179">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE179">
         <v>8000</v>
@@ -18365,7 +18365,7 @@
         <v>179</v>
       </c>
       <c r="AD180">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE180">
         <v>8000</v>
@@ -19912,7 +19912,7 @@
         <v>179</v>
       </c>
       <c r="AD196">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE196">
         <v>8000</v>
@@ -20007,7 +20007,7 @@
         <v>179</v>
       </c>
       <c r="AD197">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE197">
         <v>8000</v>
@@ -20102,7 +20102,7 @@
         <v>179</v>
       </c>
       <c r="AD198">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE198">
         <v>8000</v>
@@ -20197,7 +20197,7 @@
         <v>179</v>
       </c>
       <c r="AD199">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE199">
         <v>8000</v>
@@ -20295,7 +20295,7 @@
         <v>179</v>
       </c>
       <c r="AD200">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE200">
         <v>8000</v>
@@ -20393,7 +20393,7 @@
         <v>179</v>
       </c>
       <c r="AD201">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE201">
         <v>8000</v>
@@ -20491,7 +20491,7 @@
         <v>179</v>
       </c>
       <c r="AD202">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE202">
         <v>8000</v>
@@ -20589,7 +20589,7 @@
         <v>179</v>
       </c>
       <c r="AD203">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE203">
         <v>8000</v>
@@ -20687,7 +20687,7 @@
         <v>179</v>
       </c>
       <c r="AD204">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE204">
         <v>8000</v>
@@ -20785,7 +20785,7 @@
         <v>179</v>
       </c>
       <c r="AD205">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE205">
         <v>8000</v>
@@ -20880,7 +20880,7 @@
         <v>179</v>
       </c>
       <c r="AD206">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE206">
         <v>8000</v>
@@ -20975,7 +20975,7 @@
         <v>179</v>
       </c>
       <c r="AD207">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE207">
         <v>8000</v>
@@ -21070,7 +21070,7 @@
         <v>179</v>
       </c>
       <c r="AD208">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE208">
         <v>8000</v>
@@ -21165,7 +21165,7 @@
         <v>179</v>
       </c>
       <c r="AD209">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE209">
         <v>8000</v>
@@ -21263,7 +21263,7 @@
         <v>179</v>
       </c>
       <c r="AD210">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE210">
         <v>8000</v>
@@ -21361,7 +21361,7 @@
         <v>179</v>
       </c>
       <c r="AD211">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE211">
         <v>8000</v>
@@ -21459,7 +21459,7 @@
         <v>179</v>
       </c>
       <c r="AD212">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE212">
         <v>8000</v>
@@ -21557,7 +21557,7 @@
         <v>179</v>
       </c>
       <c r="AD213">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE213">
         <v>8000</v>
@@ -21655,7 +21655,7 @@
         <v>179</v>
       </c>
       <c r="AD214">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE214">
         <v>8000</v>
@@ -21753,7 +21753,7 @@
         <v>179</v>
       </c>
       <c r="AD215">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE215">
         <v>8000</v>
@@ -21848,7 +21848,7 @@
         <v>179</v>
       </c>
       <c r="AD216">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE216">
         <v>8000</v>
@@ -21943,7 +21943,7 @@
         <v>179</v>
       </c>
       <c r="AD217">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE217">
         <v>8000</v>
@@ -22038,7 +22038,7 @@
         <v>179</v>
       </c>
       <c r="AD218">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE218">
         <v>8000</v>
@@ -22133,7 +22133,7 @@
         <v>179</v>
       </c>
       <c r="AD219">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE219">
         <v>8000</v>
@@ -22228,7 +22228,7 @@
         <v>179</v>
       </c>
       <c r="AD220">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE220">
         <v>8000</v>
@@ -22323,7 +22323,7 @@
         <v>179</v>
       </c>
       <c r="AD221">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE221">
         <v>8000</v>
@@ -22418,7 +22418,7 @@
         <v>179</v>
       </c>
       <c r="AD222">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE222">
         <v>8000</v>
@@ -22513,7 +22513,7 @@
         <v>179</v>
       </c>
       <c r="AD223">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE223">
         <v>8000</v>
@@ -22611,7 +22611,7 @@
         <v>179</v>
       </c>
       <c r="AD224">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE224">
         <v>8000</v>
@@ -22709,7 +22709,7 @@
         <v>179</v>
       </c>
       <c r="AD225">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE225">
         <v>8000</v>
@@ -22807,7 +22807,7 @@
         <v>179</v>
       </c>
       <c r="AD226">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE226">
         <v>8000</v>
@@ -22905,7 +22905,7 @@
         <v>179</v>
       </c>
       <c r="AD227">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE227">
         <v>8000</v>
@@ -23003,7 +23003,7 @@
         <v>179</v>
       </c>
       <c r="AD228">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE228">
         <v>8000</v>
@@ -23098,7 +23098,7 @@
         <v>179</v>
       </c>
       <c r="AD229">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE229">
         <v>8000</v>
@@ -23193,7 +23193,7 @@
         <v>179</v>
       </c>
       <c r="AD230">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE230">
         <v>8000</v>
@@ -23288,7 +23288,7 @@
         <v>179</v>
       </c>
       <c r="AD231">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE231">
         <v>8000</v>
@@ -23386,7 +23386,7 @@
         <v>179</v>
       </c>
       <c r="AD232">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE232">
         <v>8000</v>
@@ -23481,7 +23481,7 @@
         <v>179</v>
       </c>
       <c r="AD233">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE233">
         <v>8000</v>
@@ -23579,7 +23579,7 @@
         <v>179</v>
       </c>
       <c r="AD234">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE234">
         <v>8000</v>
@@ -23677,7 +23677,7 @@
         <v>179</v>
       </c>
       <c r="AD235">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE235">
         <v>8000</v>
@@ -23775,7 +23775,7 @@
         <v>179</v>
       </c>
       <c r="AD236">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE236">
         <v>8000</v>
@@ -23873,7 +23873,7 @@
         <v>179</v>
       </c>
       <c r="AD237">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE237">
         <v>8000</v>
@@ -23971,7 +23971,7 @@
         <v>179</v>
       </c>
       <c r="AD238">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE238">
         <v>8000</v>
@@ -24069,7 +24069,7 @@
         <v>179</v>
       </c>
       <c r="AD239">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE239">
         <v>8000</v>
@@ -24167,7 +24167,7 @@
         <v>179</v>
       </c>
       <c r="AD240">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE240">
         <v>8000</v>
@@ -24265,7 +24265,7 @@
         <v>179</v>
       </c>
       <c r="AD241">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE241">
         <v>8000</v>
@@ -24363,7 +24363,7 @@
         <v>179</v>
       </c>
       <c r="AD242">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE242">
         <v>8000</v>
@@ -24461,7 +24461,7 @@
         <v>179</v>
       </c>
       <c r="AD243">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE243">
         <v>8000</v>
@@ -24559,7 +24559,7 @@
         <v>179</v>
       </c>
       <c r="AD244">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE244">
         <v>8000</v>
@@ -24657,7 +24657,7 @@
         <v>179</v>
       </c>
       <c r="AD245">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE245">
         <v>8000</v>
@@ -25723,7 +25723,7 @@
         <v>179</v>
       </c>
       <c r="AD256">
-        <v>10</v>
+        <v>0.2777777777777778</v>
       </c>
       <c r="AE256">
         <v>8000</v>
@@ -25821,7 +25821,7 @@
         <v>179</v>
       </c>
       <c r="AD257">
-        <v>10</v>
+        <v>0.2777777777777778</v>
       </c>
       <c r="AE257">
         <v>8000</v>
@@ -25916,7 +25916,7 @@
         <v>179</v>
       </c>
       <c r="AD258">
-        <v>10</v>
+        <v>0.2777777777777778</v>
       </c>
       <c r="AE258">
         <v>8000</v>
@@ -26011,7 +26011,7 @@
         <v>179</v>
       </c>
       <c r="AD259">
-        <v>10</v>
+        <v>0.2777777777777778</v>
       </c>
       <c r="AE259">
         <v>8000</v>
@@ -26109,7 +26109,7 @@
         <v>179</v>
       </c>
       <c r="AD260">
-        <v>10</v>
+        <v>0.2777777777777778</v>
       </c>
       <c r="AE260">
         <v>8000</v>
@@ -27175,7 +27175,7 @@
         <v>179</v>
       </c>
       <c r="AD271">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE271">
         <v>8000</v>
@@ -27273,7 +27273,7 @@
         <v>179</v>
       </c>
       <c r="AD272">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE272">
         <v>8000</v>
@@ -27371,7 +27371,7 @@
         <v>179</v>
       </c>
       <c r="AD273">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE273">
         <v>8000</v>
@@ -27466,7 +27466,7 @@
         <v>179</v>
       </c>
       <c r="AD274">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE274">
         <v>8000</v>
@@ -27561,7 +27561,7 @@
         <v>179</v>
       </c>
       <c r="AD275">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE275">
         <v>8000</v>
@@ -27656,7 +27656,7 @@
         <v>179</v>
       </c>
       <c r="AD276">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE276">
         <v>8000</v>
@@ -27751,7 +27751,7 @@
         <v>179</v>
       </c>
       <c r="AD277">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE277">
         <v>8000</v>
@@ -27849,7 +27849,7 @@
         <v>179</v>
       </c>
       <c r="AD278">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE278">
         <v>8000</v>
@@ -27947,7 +27947,7 @@
         <v>179</v>
       </c>
       <c r="AD279">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE279">
         <v>8000</v>
@@ -28042,7 +28042,7 @@
         <v>179</v>
       </c>
       <c r="AD280">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE280">
         <v>8000</v>
@@ -28137,7 +28137,7 @@
         <v>179</v>
       </c>
       <c r="AD281">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE281">
         <v>8000</v>
@@ -28235,7 +28235,7 @@
         <v>179</v>
       </c>
       <c r="AD282">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE282">
         <v>8000</v>
@@ -28330,7 +28330,7 @@
         <v>179</v>
       </c>
       <c r="AD283">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE283">
         <v>8000</v>
@@ -28425,7 +28425,7 @@
         <v>179</v>
       </c>
       <c r="AD284">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE284">
         <v>8000</v>
@@ -28523,7 +28523,7 @@
         <v>179</v>
       </c>
       <c r="AD285">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE285">
         <v>8000</v>
@@ -28621,7 +28621,7 @@
         <v>179</v>
       </c>
       <c r="AD286">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE286">
         <v>8000</v>
@@ -28719,7 +28719,7 @@
         <v>179</v>
       </c>
       <c r="AD287">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE287">
         <v>8000</v>
@@ -28817,7 +28817,7 @@
         <v>179</v>
       </c>
       <c r="AD288">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE288">
         <v>8000</v>
@@ -28915,7 +28915,7 @@
         <v>179</v>
       </c>
       <c r="AD289">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE289">
         <v>8000</v>
@@ -29010,7 +29010,7 @@
         <v>179</v>
       </c>
       <c r="AD290">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE290">
         <v>8000</v>
@@ -29105,7 +29105,7 @@
         <v>179</v>
       </c>
       <c r="AD291">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE291">
         <v>8000</v>
@@ -29203,7 +29203,7 @@
         <v>179</v>
       </c>
       <c r="AD292">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE292">
         <v>8000</v>
@@ -29301,7 +29301,7 @@
         <v>179</v>
       </c>
       <c r="AD293">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE293">
         <v>8000</v>
@@ -29399,7 +29399,7 @@
         <v>179</v>
       </c>
       <c r="AD294">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE294">
         <v>8000</v>
@@ -29497,7 +29497,7 @@
         <v>179</v>
       </c>
       <c r="AD295">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE295">
         <v>8000</v>
@@ -34916,7 +34916,7 @@
         <v>179</v>
       </c>
       <c r="AD351">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE351">
         <v>8000</v>
@@ -35011,7 +35011,7 @@
         <v>179</v>
       </c>
       <c r="AD352">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE352">
         <v>8000</v>
@@ -35106,7 +35106,7 @@
         <v>179</v>
       </c>
       <c r="AD353">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE353">
         <v>8000</v>
@@ -35201,7 +35201,7 @@
         <v>179</v>
       </c>
       <c r="AD354">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE354">
         <v>8000</v>
@@ -35296,7 +35296,7 @@
         <v>179</v>
       </c>
       <c r="AD355">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE355">
         <v>8000</v>
@@ -35391,7 +35391,7 @@
         <v>179</v>
       </c>
       <c r="AD356">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE356">
         <v>8000</v>
@@ -35486,7 +35486,7 @@
         <v>179</v>
       </c>
       <c r="AD357">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE357">
         <v>8000</v>
@@ -35584,7 +35584,7 @@
         <v>179</v>
       </c>
       <c r="AD358">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE358">
         <v>8000</v>
@@ -35682,7 +35682,7 @@
         <v>179</v>
       </c>
       <c r="AD359">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE359">
         <v>8000</v>
@@ -35780,7 +35780,7 @@
         <v>179</v>
       </c>
       <c r="AD360">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE360">
         <v>8000</v>
@@ -35878,7 +35878,7 @@
         <v>179</v>
       </c>
       <c r="AD361">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE361">
         <v>8000</v>
@@ -35976,7 +35976,7 @@
         <v>179</v>
       </c>
       <c r="AD362">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE362">
         <v>8000</v>
@@ -36074,7 +36074,7 @@
         <v>179</v>
       </c>
       <c r="AD363">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE363">
         <v>8000</v>
@@ -36172,7 +36172,7 @@
         <v>179</v>
       </c>
       <c r="AD364">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE364">
         <v>8000</v>
@@ -36270,7 +36270,7 @@
         <v>179</v>
       </c>
       <c r="AD365">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE365">
         <v>8000</v>
@@ -36368,7 +36368,7 @@
         <v>179</v>
       </c>
       <c r="AD366">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE366">
         <v>8000</v>
@@ -36466,7 +36466,7 @@
         <v>179</v>
       </c>
       <c r="AD367">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE367">
         <v>8000</v>
@@ -36561,7 +36561,7 @@
         <v>179</v>
       </c>
       <c r="AD368">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE368">
         <v>8000</v>
@@ -36656,7 +36656,7 @@
         <v>179</v>
       </c>
       <c r="AD369">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE369">
         <v>8000</v>
@@ -36754,7 +36754,7 @@
         <v>179</v>
       </c>
       <c r="AD370">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE370">
         <v>8000</v>
@@ -36852,7 +36852,7 @@
         <v>179</v>
       </c>
       <c r="AD371">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE371">
         <v>8000</v>
@@ -36950,7 +36950,7 @@
         <v>179</v>
       </c>
       <c r="AD372">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE372">
         <v>8000</v>
@@ -37048,7 +37048,7 @@
         <v>179</v>
       </c>
       <c r="AD373">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE373">
         <v>8000</v>
@@ -37146,7 +37146,7 @@
         <v>179</v>
       </c>
       <c r="AD374">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE374">
         <v>8000</v>
@@ -37244,7 +37244,7 @@
         <v>179</v>
       </c>
       <c r="AD375">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE375">
         <v>8000</v>
@@ -37342,7 +37342,7 @@
         <v>179</v>
       </c>
       <c r="AD376">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE376">
         <v>8000</v>
@@ -37440,7 +37440,7 @@
         <v>179</v>
       </c>
       <c r="AD377">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE377">
         <v>8000</v>
@@ -37538,7 +37538,7 @@
         <v>179</v>
       </c>
       <c r="AD378">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE378">
         <v>8000</v>
@@ -37636,7 +37636,7 @@
         <v>179</v>
       </c>
       <c r="AD379">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE379">
         <v>8000</v>
@@ -37734,7 +37734,7 @@
         <v>179</v>
       </c>
       <c r="AD380">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE380">
         <v>8000</v>
@@ -37832,7 +37832,7 @@
         <v>179</v>
       </c>
       <c r="AD381">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE381">
         <v>8000</v>
@@ -37927,7 +37927,7 @@
         <v>179</v>
       </c>
       <c r="AD382">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE382">
         <v>8000</v>
@@ -38022,7 +38022,7 @@
         <v>179</v>
       </c>
       <c r="AD383">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE383">
         <v>8000</v>
@@ -38117,7 +38117,7 @@
         <v>179</v>
       </c>
       <c r="AD384">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE384">
         <v>8000</v>
@@ -38212,7 +38212,7 @@
         <v>179</v>
       </c>
       <c r="AD385">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE385">
         <v>8000</v>
@@ -38307,7 +38307,7 @@
         <v>179</v>
       </c>
       <c r="AD386">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE386">
         <v>8000</v>
@@ -38405,7 +38405,7 @@
         <v>179</v>
       </c>
       <c r="AD387">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE387">
         <v>8000</v>
@@ -38500,7 +38500,7 @@
         <v>179</v>
       </c>
       <c r="AD388">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE388">
         <v>8000</v>
@@ -38598,7 +38598,7 @@
         <v>179</v>
       </c>
       <c r="AD389">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE389">
         <v>8000</v>
@@ -38696,7 +38696,7 @@
         <v>179</v>
       </c>
       <c r="AD390">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE390">
         <v>8000</v>
@@ -38794,7 +38794,7 @@
         <v>179</v>
       </c>
       <c r="AD391">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE391">
         <v>8000</v>
@@ -38892,7 +38892,7 @@
         <v>179</v>
       </c>
       <c r="AD392">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE392">
         <v>8000</v>
@@ -38990,7 +38990,7 @@
         <v>179</v>
       </c>
       <c r="AD393">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE393">
         <v>8000</v>
@@ -39085,7 +39085,7 @@
         <v>179</v>
       </c>
       <c r="AD394">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE394">
         <v>8000</v>
@@ -39183,7 +39183,7 @@
         <v>179</v>
       </c>
       <c r="AD395">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE395">
         <v>8000</v>
@@ -39281,7 +39281,7 @@
         <v>179</v>
       </c>
       <c r="AD396">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE396">
         <v>8000</v>
@@ -39379,7 +39379,7 @@
         <v>179</v>
       </c>
       <c r="AD397">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE397">
         <v>8000</v>
@@ -39474,7 +39474,7 @@
         <v>179</v>
       </c>
       <c r="AD398">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE398">
         <v>8000</v>
@@ -39569,7 +39569,7 @@
         <v>179</v>
       </c>
       <c r="AD399">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE399">
         <v>8000</v>
@@ -39664,7 +39664,7 @@
         <v>179</v>
       </c>
       <c r="AD400">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE400">
         <v>8000</v>
@@ -39762,7 +39762,7 @@
         <v>179</v>
       </c>
       <c r="AD401">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE401">
         <v>8000</v>
@@ -39857,7 +39857,7 @@
         <v>179</v>
       </c>
       <c r="AD402">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE402">
         <v>8000</v>
@@ -39952,7 +39952,7 @@
         <v>179</v>
       </c>
       <c r="AD403">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE403">
         <v>8000</v>
@@ -40050,7 +40050,7 @@
         <v>179</v>
       </c>
       <c r="AD404">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE404">
         <v>8000</v>
@@ -40145,7 +40145,7 @@
         <v>179</v>
       </c>
       <c r="AD405">
-        <v>10</v>
+        <v>12.93898809523811</v>
       </c>
       <c r="AE405">
         <v>8000</v>
@@ -40243,7 +40243,7 @@
         <v>179</v>
       </c>
       <c r="AD406">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE406">
         <v>8000</v>
@@ -40341,7 +40341,7 @@
         <v>179</v>
       </c>
       <c r="AD407">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE407">
         <v>8000</v>
@@ -40439,7 +40439,7 @@
         <v>179</v>
       </c>
       <c r="AD408">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE408">
         <v>8000</v>
@@ -40534,7 +40534,7 @@
         <v>179</v>
       </c>
       <c r="AD409">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE409">
         <v>8000</v>
@@ -40629,7 +40629,7 @@
         <v>179</v>
       </c>
       <c r="AD410">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE410">
         <v>8000</v>
@@ -40724,7 +40724,7 @@
         <v>179</v>
       </c>
       <c r="AD411">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE411">
         <v>8000</v>
@@ -40819,7 +40819,7 @@
         <v>179</v>
       </c>
       <c r="AD412">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE412">
         <v>8000</v>
@@ -40914,7 +40914,7 @@
         <v>179</v>
       </c>
       <c r="AD413">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE413">
         <v>8000</v>
@@ -41012,7 +41012,7 @@
         <v>179</v>
       </c>
       <c r="AD414">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE414">
         <v>8000</v>
@@ -41110,7 +41110,7 @@
         <v>179</v>
       </c>
       <c r="AD415">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE415">
         <v>8000</v>
@@ -41205,7 +41205,7 @@
         <v>179</v>
       </c>
       <c r="AD416">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE416">
         <v>8000</v>
@@ -41303,7 +41303,7 @@
         <v>179</v>
       </c>
       <c r="AD417">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE417">
         <v>8000</v>
@@ -41401,7 +41401,7 @@
         <v>179</v>
       </c>
       <c r="AD418">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE418">
         <v>8000</v>
@@ -41499,7 +41499,7 @@
         <v>179</v>
       </c>
       <c r="AD419">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE419">
         <v>8000</v>
@@ -41597,7 +41597,7 @@
         <v>179</v>
       </c>
       <c r="AD420">
-        <v>10</v>
+        <v>13.76976495726495</v>
       </c>
       <c r="AE420">
         <v>8000</v>
@@ -41692,7 +41692,7 @@
         <v>179</v>
       </c>
       <c r="AD421">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE421">
         <v>8000</v>
@@ -41787,7 +41787,7 @@
         <v>179</v>
       </c>
       <c r="AD422">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE422">
         <v>8000</v>
@@ -41882,7 +41882,7 @@
         <v>179</v>
       </c>
       <c r="AD423">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE423">
         <v>8000</v>
@@ -41977,7 +41977,7 @@
         <v>179</v>
       </c>
       <c r="AD424">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE424">
         <v>8000</v>
@@ -42075,7 +42075,7 @@
         <v>179</v>
       </c>
       <c r="AD425">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE425">
         <v>8000</v>
@@ -42170,7 +42170,7 @@
         <v>179</v>
       </c>
       <c r="AD426">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE426">
         <v>8000</v>
@@ -42265,7 +42265,7 @@
         <v>179</v>
       </c>
       <c r="AD427">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE427">
         <v>8000</v>
@@ -42363,7 +42363,7 @@
         <v>179</v>
       </c>
       <c r="AD428">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE428">
         <v>8000</v>
@@ -42458,7 +42458,7 @@
         <v>179</v>
       </c>
       <c r="AD429">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE429">
         <v>8000</v>
@@ -42553,7 +42553,7 @@
         <v>179</v>
       </c>
       <c r="AD430">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE430">
         <v>8000</v>
@@ -42651,7 +42651,7 @@
         <v>179</v>
       </c>
       <c r="AD431">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE431">
         <v>8000</v>
@@ -42749,7 +42749,7 @@
         <v>179</v>
       </c>
       <c r="AD432">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE432">
         <v>8000</v>
@@ -42847,7 +42847,7 @@
         <v>179</v>
       </c>
       <c r="AD433">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE433">
         <v>8000</v>
@@ -42945,7 +42945,7 @@
         <v>179</v>
       </c>
       <c r="AD434">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE434">
         <v>8000</v>
@@ -43040,7 +43040,7 @@
         <v>179</v>
       </c>
       <c r="AD435">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE435">
         <v>8000</v>
@@ -43138,7 +43138,7 @@
         <v>179</v>
       </c>
       <c r="AD436">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE436">
         <v>8000</v>
@@ -43236,7 +43236,7 @@
         <v>179</v>
       </c>
       <c r="AD437">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE437">
         <v>8000</v>
@@ -43334,7 +43334,7 @@
         <v>179</v>
       </c>
       <c r="AD438">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE438">
         <v>8000</v>
@@ -43432,7 +43432,7 @@
         <v>179</v>
       </c>
       <c r="AD439">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE439">
         <v>8000</v>
@@ -43530,7 +43530,7 @@
         <v>179</v>
       </c>
       <c r="AD440">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE440">
         <v>8000</v>
@@ -43628,7 +43628,7 @@
         <v>179</v>
       </c>
       <c r="AD441">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE441">
         <v>8000</v>
@@ -43726,7 +43726,7 @@
         <v>179</v>
       </c>
       <c r="AD442">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE442">
         <v>8000</v>
@@ -43824,7 +43824,7 @@
         <v>179</v>
       </c>
       <c r="AD443">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE443">
         <v>8000</v>
@@ -43922,7 +43922,7 @@
         <v>179</v>
       </c>
       <c r="AD444">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE444">
         <v>8000</v>
@@ -44020,7 +44020,7 @@
         <v>179</v>
       </c>
       <c r="AD445">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE445">
         <v>8000</v>
@@ -44118,7 +44118,7 @@
         <v>179</v>
       </c>
       <c r="AD446">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE446">
         <v>8000</v>
@@ -44216,7 +44216,7 @@
         <v>179</v>
       </c>
       <c r="AD447">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE447">
         <v>8000</v>
@@ -44314,7 +44314,7 @@
         <v>179</v>
       </c>
       <c r="AD448">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE448">
         <v>8000</v>
@@ -44412,7 +44412,7 @@
         <v>179</v>
       </c>
       <c r="AD449">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE449">
         <v>8000</v>
@@ -44510,7 +44510,7 @@
         <v>179</v>
       </c>
       <c r="AD450">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE450">
         <v>8000</v>
@@ -44608,7 +44608,7 @@
         <v>179</v>
       </c>
       <c r="AD451">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE451">
         <v>8000</v>
@@ -44703,7 +44703,7 @@
         <v>179</v>
       </c>
       <c r="AD452">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE452">
         <v>8000</v>
@@ -44801,7 +44801,7 @@
         <v>179</v>
       </c>
       <c r="AD453">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE453">
         <v>8000</v>
@@ -44899,7 +44899,7 @@
         <v>179</v>
       </c>
       <c r="AD454">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE454">
         <v>8000</v>
@@ -44997,7 +44997,7 @@
         <v>179</v>
       </c>
       <c r="AD455">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE455">
         <v>8000</v>
@@ -45095,7 +45095,7 @@
         <v>179</v>
       </c>
       <c r="AD456">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE456">
         <v>8000</v>
@@ -45193,7 +45193,7 @@
         <v>179</v>
       </c>
       <c r="AD457">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE457">
         <v>8000</v>
@@ -45288,7 +45288,7 @@
         <v>179</v>
       </c>
       <c r="AD458">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE458">
         <v>8000</v>
@@ -45383,7 +45383,7 @@
         <v>179</v>
       </c>
       <c r="AD459">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE459">
         <v>8000</v>
@@ -45478,7 +45478,7 @@
         <v>179</v>
       </c>
       <c r="AD460">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE460">
         <v>8000</v>
@@ -45573,7 +45573,7 @@
         <v>179</v>
       </c>
       <c r="AD461">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE461">
         <v>8000</v>
@@ -45668,7 +45668,7 @@
         <v>179</v>
       </c>
       <c r="AD462">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE462">
         <v>8000</v>
@@ -45763,7 +45763,7 @@
         <v>179</v>
       </c>
       <c r="AD463">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE463">
         <v>8000</v>
@@ -45858,7 +45858,7 @@
         <v>179</v>
       </c>
       <c r="AD464">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE464">
         <v>8000</v>
@@ -45953,7 +45953,7 @@
         <v>179</v>
       </c>
       <c r="AD465">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE465">
         <v>8000</v>
@@ -46051,7 +46051,7 @@
         <v>179</v>
       </c>
       <c r="AD466">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE466">
         <v>8000</v>
@@ -46149,7 +46149,7 @@
         <v>179</v>
       </c>
       <c r="AD467">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE467">
         <v>8000</v>
@@ -46247,7 +46247,7 @@
         <v>179</v>
       </c>
       <c r="AD468">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE468">
         <v>8000</v>
@@ -46345,7 +46345,7 @@
         <v>179</v>
       </c>
       <c r="AD469">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE469">
         <v>8000</v>
@@ -46443,7 +46443,7 @@
         <v>179</v>
       </c>
       <c r="AD470">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE470">
         <v>8000</v>
@@ -46541,7 +46541,7 @@
         <v>179</v>
       </c>
       <c r="AD471">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE471">
         <v>8000</v>
@@ -46639,7 +46639,7 @@
         <v>179</v>
       </c>
       <c r="AD472">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE472">
         <v>8000</v>
@@ -46734,7 +46734,7 @@
         <v>179</v>
       </c>
       <c r="AD473">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE473">
         <v>8000</v>
@@ -46829,7 +46829,7 @@
         <v>179</v>
       </c>
       <c r="AD474">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE474">
         <v>8000</v>
@@ -46924,7 +46924,7 @@
         <v>179</v>
       </c>
       <c r="AD475">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE475">
         <v>8000</v>
@@ -47019,7 +47019,7 @@
         <v>179</v>
       </c>
       <c r="AD476">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE476">
         <v>8000</v>
@@ -47117,7 +47117,7 @@
         <v>179</v>
       </c>
       <c r="AD477">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE477">
         <v>8000</v>
@@ -47215,7 +47215,7 @@
         <v>179</v>
       </c>
       <c r="AD478">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE478">
         <v>8000</v>
@@ -47313,7 +47313,7 @@
         <v>179</v>
       </c>
       <c r="AD479">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE479">
         <v>8000</v>
@@ -47411,7 +47411,7 @@
         <v>179</v>
       </c>
       <c r="AD480">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE480">
         <v>8000</v>
@@ -47509,7 +47509,7 @@
         <v>179</v>
       </c>
       <c r="AD481">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE481">
         <v>8000</v>
@@ -47607,7 +47607,7 @@
         <v>179</v>
       </c>
       <c r="AD482">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE482">
         <v>8000</v>
@@ -47705,7 +47705,7 @@
         <v>179</v>
       </c>
       <c r="AD483">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE483">
         <v>8000</v>
@@ -47803,7 +47803,7 @@
         <v>179</v>
       </c>
       <c r="AD484">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE484">
         <v>8000</v>
@@ -47901,7 +47901,7 @@
         <v>179</v>
       </c>
       <c r="AD485">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE485">
         <v>8000</v>
@@ -47999,7 +47999,7 @@
         <v>179</v>
       </c>
       <c r="AD486">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE486">
         <v>8000</v>
@@ -48097,7 +48097,7 @@
         <v>179</v>
       </c>
       <c r="AD487">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE487">
         <v>8000</v>
@@ -48195,7 +48195,7 @@
         <v>179</v>
       </c>
       <c r="AD488">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE488">
         <v>8000</v>
@@ -48293,7 +48293,7 @@
         <v>179</v>
       </c>
       <c r="AD489">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE489">
         <v>8000</v>
@@ -48391,7 +48391,7 @@
         <v>179</v>
       </c>
       <c r="AD490">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE490">
         <v>8000</v>
@@ -48489,7 +48489,7 @@
         <v>179</v>
       </c>
       <c r="AD491">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE491">
         <v>8000</v>
@@ -48587,7 +48587,7 @@
         <v>179</v>
       </c>
       <c r="AD492">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE492">
         <v>8000</v>
@@ -48682,7 +48682,7 @@
         <v>179</v>
       </c>
       <c r="AD493">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE493">
         <v>8000</v>
@@ -48777,7 +48777,7 @@
         <v>179</v>
       </c>
       <c r="AD494">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE494">
         <v>8000</v>
@@ -48875,7 +48875,7 @@
         <v>179</v>
       </c>
       <c r="AD495">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE495">
         <v>8000</v>
@@ -48973,7 +48973,7 @@
         <v>179</v>
       </c>
       <c r="AD496">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE496">
         <v>8000</v>
@@ -49071,7 +49071,7 @@
         <v>179</v>
       </c>
       <c r="AD497">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE497">
         <v>8000</v>
@@ -49169,7 +49169,7 @@
         <v>179</v>
       </c>
       <c r="AD498">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE498">
         <v>8000</v>
@@ -49267,7 +49267,7 @@
         <v>179</v>
       </c>
       <c r="AD499">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE499">
         <v>8000</v>
@@ -49365,7 +49365,7 @@
         <v>179</v>
       </c>
       <c r="AD500">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE500">
         <v>8000</v>
@@ -49463,7 +49463,7 @@
         <v>179</v>
       </c>
       <c r="AD501">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE501">
         <v>8000</v>
@@ -49561,7 +49561,7 @@
         <v>179</v>
       </c>
       <c r="AD502">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE502">
         <v>8000</v>
@@ -49659,7 +49659,7 @@
         <v>179</v>
       </c>
       <c r="AD503">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE503">
         <v>8000</v>
@@ -49757,7 +49757,7 @@
         <v>179</v>
       </c>
       <c r="AD504">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE504">
         <v>8000</v>
@@ -49855,7 +49855,7 @@
         <v>179</v>
       </c>
       <c r="AD505">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE505">
         <v>8000</v>
@@ -49953,7 +49953,7 @@
         <v>179</v>
       </c>
       <c r="AD506">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE506">
         <v>8000</v>
@@ -50051,7 +50051,7 @@
         <v>179</v>
       </c>
       <c r="AD507">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE507">
         <v>8000</v>
@@ -50146,7 +50146,7 @@
         <v>179</v>
       </c>
       <c r="AD508">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE508">
         <v>8000</v>
@@ -50241,7 +50241,7 @@
         <v>179</v>
       </c>
       <c r="AD509">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE509">
         <v>8000</v>
@@ -50336,7 +50336,7 @@
         <v>179</v>
       </c>
       <c r="AD510">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE510">
         <v>8000</v>
@@ -50431,7 +50431,7 @@
         <v>179</v>
       </c>
       <c r="AD511">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE511">
         <v>8000</v>
@@ -50526,7 +50526,7 @@
         <v>179</v>
       </c>
       <c r="AD512">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE512">
         <v>8000</v>
@@ -50624,7 +50624,7 @@
         <v>179</v>
       </c>
       <c r="AD513">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE513">
         <v>8000</v>
@@ -50722,7 +50722,7 @@
         <v>179</v>
       </c>
       <c r="AD514">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE514">
         <v>8000</v>
@@ -50820,7 +50820,7 @@
         <v>179</v>
       </c>
       <c r="AD515">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE515">
         <v>8000</v>
@@ -50918,7 +50918,7 @@
         <v>179</v>
       </c>
       <c r="AD516">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE516">
         <v>8000</v>
@@ -51016,7 +51016,7 @@
         <v>179</v>
       </c>
       <c r="AD517">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE517">
         <v>8000</v>
@@ -51111,7 +51111,7 @@
         <v>179</v>
       </c>
       <c r="AD518">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE518">
         <v>8000</v>
@@ -51206,7 +51206,7 @@
         <v>179</v>
       </c>
       <c r="AD519">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE519">
         <v>8000</v>
@@ -51301,7 +51301,7 @@
         <v>179</v>
       </c>
       <c r="AD520">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE520">
         <v>8000</v>
@@ -51399,7 +51399,7 @@
         <v>179</v>
       </c>
       <c r="AD521">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE521">
         <v>8000</v>
@@ -51494,7 +51494,7 @@
         <v>179</v>
       </c>
       <c r="AD522">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE522">
         <v>8000</v>
@@ -51592,7 +51592,7 @@
         <v>179</v>
       </c>
       <c r="AD523">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE523">
         <v>8000</v>
@@ -51690,7 +51690,7 @@
         <v>179</v>
       </c>
       <c r="AD524">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE524">
         <v>8000</v>
@@ -51788,7 +51788,7 @@
         <v>179</v>
       </c>
       <c r="AD525">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE525">
         <v>8000</v>
@@ -51886,7 +51886,7 @@
         <v>179</v>
       </c>
       <c r="AD526">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE526">
         <v>8000</v>
@@ -51984,7 +51984,7 @@
         <v>179</v>
       </c>
       <c r="AD527">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE527">
         <v>8000</v>
@@ -52082,7 +52082,7 @@
         <v>179</v>
       </c>
       <c r="AD528">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE528">
         <v>8000</v>
@@ -52177,7 +52177,7 @@
         <v>179</v>
       </c>
       <c r="AD529">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE529">
         <v>8000</v>
@@ -52272,7 +52272,7 @@
         <v>179</v>
       </c>
       <c r="AD530">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE530">
         <v>8000</v>
@@ -52367,7 +52367,7 @@
         <v>179</v>
       </c>
       <c r="AD531">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE531">
         <v>8000</v>
@@ -52462,7 +52462,7 @@
         <v>179</v>
       </c>
       <c r="AD532">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE532">
         <v>8000</v>
@@ -52557,7 +52557,7 @@
         <v>179</v>
       </c>
       <c r="AD533">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE533">
         <v>8000</v>
@@ -52652,7 +52652,7 @@
         <v>179</v>
       </c>
       <c r="AD534">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE534">
         <v>8000</v>
@@ -52747,7 +52747,7 @@
         <v>179</v>
       </c>
       <c r="AD535">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE535">
         <v>8000</v>
@@ -52842,7 +52842,7 @@
         <v>179</v>
       </c>
       <c r="AD536">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE536">
         <v>8000</v>
@@ -52937,7 +52937,7 @@
         <v>179</v>
       </c>
       <c r="AD537">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE537">
         <v>8000</v>
@@ -53032,7 +53032,7 @@
         <v>179</v>
       </c>
       <c r="AD538">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE538">
         <v>8000</v>
@@ -53127,7 +53127,7 @@
         <v>179</v>
       </c>
       <c r="AD539">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE539">
         <v>8000</v>
@@ -53222,7 +53222,7 @@
         <v>179</v>
       </c>
       <c r="AD540">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE540">
         <v>8000</v>
@@ -53317,7 +53317,7 @@
         <v>179</v>
       </c>
       <c r="AD541">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE541">
         <v>8000</v>
@@ -53412,7 +53412,7 @@
         <v>179</v>
       </c>
       <c r="AD542">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE542">
         <v>8000</v>
@@ -53507,7 +53507,7 @@
         <v>179</v>
       </c>
       <c r="AD543">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE543">
         <v>8000</v>
@@ -53602,7 +53602,7 @@
         <v>179</v>
       </c>
       <c r="AD544">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE544">
         <v>8000</v>
@@ -53697,7 +53697,7 @@
         <v>179</v>
       </c>
       <c r="AD545">
-        <v>10</v>
+        <v>5.462962962962945</v>
       </c>
       <c r="AE545">
         <v>8000</v>
@@ -53795,7 +53795,7 @@
         <v>179</v>
       </c>
       <c r="AD546">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE546">
         <v>8000</v>
@@ -53893,7 +53893,7 @@
         <v>179</v>
       </c>
       <c r="AD547">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE547">
         <v>8000</v>
@@ -53991,7 +53991,7 @@
         <v>179</v>
       </c>
       <c r="AD548">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE548">
         <v>8000</v>
@@ -54086,7 +54086,7 @@
         <v>179</v>
       </c>
       <c r="AD549">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE549">
         <v>8000</v>
@@ -54184,7 +54184,7 @@
         <v>179</v>
       </c>
       <c r="AD550">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE550">
         <v>8000</v>
@@ -54279,7 +54279,7 @@
         <v>179</v>
       </c>
       <c r="AD551">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE551">
         <v>8000</v>
@@ -54374,7 +54374,7 @@
         <v>179</v>
       </c>
       <c r="AD552">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE552">
         <v>8000</v>
@@ -54469,7 +54469,7 @@
         <v>179</v>
       </c>
       <c r="AD553">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE553">
         <v>8000</v>
@@ -54567,7 +54567,7 @@
         <v>179</v>
       </c>
       <c r="AD554">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE554">
         <v>8000</v>
@@ -54665,7 +54665,7 @@
         <v>179</v>
       </c>
       <c r="AD555">
-        <v>10</v>
+        <v>19.60879629629628</v>
       </c>
       <c r="AE555">
         <v>8000</v>
@@ -54763,7 +54763,7 @@
         <v>179</v>
       </c>
       <c r="AD556">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE556">
         <v>8000</v>
@@ -54861,7 +54861,7 @@
         <v>179</v>
       </c>
       <c r="AD557">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE557">
         <v>8000</v>
@@ -54959,7 +54959,7 @@
         <v>179</v>
       </c>
       <c r="AD558">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE558">
         <v>8000</v>
@@ -55057,7 +55057,7 @@
         <v>179</v>
       </c>
       <c r="AD559">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE559">
         <v>8000</v>
@@ -55155,7 +55155,7 @@
         <v>179</v>
       </c>
       <c r="AD560">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE560">
         <v>8000</v>
@@ -55250,7 +55250,7 @@
         <v>179</v>
       </c>
       <c r="AD561">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE561">
         <v>8000</v>
@@ -55348,7 +55348,7 @@
         <v>179</v>
       </c>
       <c r="AD562">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE562">
         <v>8000</v>
@@ -55443,7 +55443,7 @@
         <v>179</v>
       </c>
       <c r="AD563">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE563">
         <v>8000</v>
@@ -55538,7 +55538,7 @@
         <v>179</v>
       </c>
       <c r="AD564">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE564">
         <v>8000</v>
@@ -55633,7 +55633,7 @@
         <v>179</v>
       </c>
       <c r="AD565">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE565">
         <v>8000</v>
@@ -55731,7 +55731,7 @@
         <v>179</v>
       </c>
       <c r="AD566">
-        <v>10</v>
+        <v>21.28240740740739</v>
       </c>
       <c r="AE566">
         <v>8000</v>
@@ -55829,7 +55829,7 @@
         <v>179</v>
       </c>
       <c r="AD567">
-        <v>10</v>
+        <v>21.28240740740739</v>
       </c>
       <c r="AE567">
         <v>8000</v>
@@ -55924,7 +55924,7 @@
         <v>179</v>
       </c>
       <c r="AD568">
-        <v>10</v>
+        <v>21.28240740740739</v>
       </c>
       <c r="AE568">
         <v>8000</v>
@@ -56022,7 +56022,7 @@
         <v>179</v>
       </c>
       <c r="AD569">
-        <v>10</v>
+        <v>21.28240740740739</v>
       </c>
       <c r="AE569">
         <v>8000</v>
@@ -56120,7 +56120,7 @@
         <v>179</v>
       </c>
       <c r="AD570">
-        <v>10</v>
+        <v>21.28240740740739</v>
       </c>
       <c r="AE570">
         <v>8000</v>
@@ -56215,7 +56215,7 @@
         <v>179</v>
       </c>
       <c r="AD571">
-        <v>10</v>
+        <v>21.28240740740739</v>
       </c>
       <c r="AE571">
         <v>8000</v>
@@ -56313,7 +56313,7 @@
         <v>179</v>
       </c>
       <c r="AD572">
-        <v>10</v>
+        <v>21.28240740740739</v>
       </c>
       <c r="AE572">
         <v>8000</v>
@@ -56408,7 +56408,7 @@
         <v>179</v>
       </c>
       <c r="AD573">
-        <v>10</v>
+        <v>21.28240740740739</v>
       </c>
       <c r="AE573">
         <v>8000</v>
@@ -56506,7 +56506,7 @@
         <v>179</v>
       </c>
       <c r="AD574">
-        <v>10</v>
+        <v>21.28240740740739</v>
       </c>
       <c r="AE574">
         <v>8000</v>
@@ -56601,7 +56601,7 @@
         <v>179</v>
       </c>
       <c r="AD575">
-        <v>10</v>
+        <v>21.28240740740739</v>
       </c>
       <c r="AE575">
         <v>8000</v>
@@ -56699,7 +56699,7 @@
         <v>179</v>
       </c>
       <c r="AD576">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE576">
         <v>8000</v>
@@ -56797,7 +56797,7 @@
         <v>179</v>
       </c>
       <c r="AD577">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE577">
         <v>8000</v>
@@ -56895,7 +56895,7 @@
         <v>179</v>
       </c>
       <c r="AD578">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE578">
         <v>8000</v>
@@ -56993,7 +56993,7 @@
         <v>179</v>
       </c>
       <c r="AD579">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE579">
         <v>8000</v>
@@ -57091,7 +57091,7 @@
         <v>179</v>
       </c>
       <c r="AD580">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE580">
         <v>8000</v>
@@ -57186,7 +57186,7 @@
         <v>179</v>
       </c>
       <c r="AD581">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE581">
         <v>8000</v>
@@ -57284,7 +57284,7 @@
         <v>179</v>
       </c>
       <c r="AD582">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE582">
         <v>8000</v>
@@ -57379,7 +57379,7 @@
         <v>179</v>
       </c>
       <c r="AD583">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE583">
         <v>8000</v>
@@ -57474,7 +57474,7 @@
         <v>179</v>
       </c>
       <c r="AD584">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE584">
         <v>8000</v>
@@ -57569,7 +57569,7 @@
         <v>179</v>
       </c>
       <c r="AD585">
-        <v>10</v>
+        <v>14.47727272727272</v>
       </c>
       <c r="AE585">
         <v>8000</v>

</xml_diff>